<commit_message>
added full updated flow
</commit_message>
<xml_diff>
--- a/addresses/good_addresses.xlsx
+++ b/addresses/good_addresses.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\routecraft\addresses\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDA82F44-96F8-4D6D-95C4-07285B0D0F89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="82">
   <si>
     <t>City</t>
   </si>
@@ -112,111 +111,171 @@
     <t>41</t>
   </si>
   <si>
-    <t>משך חכמה</t>
-  </si>
-  <si>
-    <t>64</t>
-  </si>
-  <si>
-    <t>חפץ חיים</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>מסילת יוסף</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>רחוב עקיבא</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>שאגת אריה</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>רב ושמואל</t>
-  </si>
-  <si>
-    <t>עיון התלמוד</t>
-  </si>
-  <si>
-    <t>רשבא</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>חתם סופר</t>
-  </si>
-  <si>
-    <t>הבעל שם טוב</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>קהילות יעקב</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>שדרות יחזקאל</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>מרומי שדה</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>אורח חיים</t>
-  </si>
-  <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>פונוביז</t>
-  </si>
-  <si>
-    <t>נתיבות המשפט</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>חזון דוד</t>
-  </si>
-  <si>
-    <t>2</t>
+    <t>לוד</t>
+  </si>
+  <si>
+    <t xml:space="preserve">יחד שבטי ישראל </t>
+  </si>
+  <si>
+    <t xml:space="preserve">משה רבינו </t>
+  </si>
+  <si>
+    <t xml:space="preserve">השייטת </t>
+  </si>
+  <si>
+    <t xml:space="preserve">צמח צדק </t>
+  </si>
+  <si>
+    <t xml:space="preserve">שבט יהודה </t>
+  </si>
+  <si>
+    <t xml:space="preserve">שבט אשר </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> שבט יהודה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אחיסמך רבקה אימנו </t>
+  </si>
+  <si>
+    <t xml:space="preserve">שבט זבולון </t>
+  </si>
+  <si>
+    <t>עפולה</t>
+  </si>
+  <si>
+    <t>קונטיקט 5</t>
+  </si>
+  <si>
+    <t>הזהבן 4</t>
+  </si>
+  <si>
+    <t>חיננית 13</t>
+  </si>
+  <si>
+    <t>חטפית 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">פנקס צבי 8 </t>
+  </si>
+  <si>
+    <t>צוקית 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הרצל 19 </t>
+  </si>
+  <si>
+    <t>עלית הנוער 8</t>
+  </si>
+  <si>
+    <t>רחוב הרצל 24</t>
+  </si>
+  <si>
+    <t>הבריגדה היהודית 11</t>
+  </si>
+  <si>
+    <t>אבן גבירול 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">זבוטינסקי 10 </t>
+  </si>
+  <si>
+    <t>הרוגי מלכות 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">עליית הנוער 9 </t>
+  </si>
+  <si>
+    <t>ראסל 10</t>
+  </si>
+  <si>
+    <t>ירקון 11</t>
+  </si>
+  <si>
+    <t>אבן גבירול 45</t>
+  </si>
+  <si>
+    <t>אבן גבירול 30</t>
+  </si>
+  <si>
+    <t>רכסים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">רחוב סביון </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הכלניות </t>
+  </si>
+  <si>
+    <t xml:space="preserve">כלניות </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הורדים  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ורדים </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הנרקיסים  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הנרקיסים </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הכלניות  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">רחוב הזית </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הדקל </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הדס </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הדס  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">אשל </t>
+  </si>
+  <si>
+    <t xml:space="preserve">דקל </t>
+  </si>
+  <si>
+    <t xml:space="preserve">השקד  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">השקד </t>
+  </si>
+  <si>
+    <t xml:space="preserve">מעלה החזון איש </t>
+  </si>
+  <si>
+    <t xml:space="preserve">חזון איש </t>
+  </si>
+  <si>
+    <t xml:space="preserve">רימונים </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הרימונים </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הרב קוק  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הרב קוק </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -224,7 +283,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -255,13 +314,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -564,13 +630,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E261"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.8984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -751,7 +817,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>3</v>
       </c>
@@ -762,7 +828,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>3</v>
       </c>
@@ -773,539 +839,846 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="D19" s="3"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="4" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="D20" s="3"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" s="4">
+        <v>46</v>
+      </c>
+      <c r="D21" s="3"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="4">
+        <v>6</v>
+      </c>
+      <c r="D22" s="3"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="4">
         <v>3</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="D23" s="3"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="B24" s="5" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="C24" s="4">
+        <v>8</v>
+      </c>
+      <c r="D24" s="3"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C25" s="4">
+        <v>5</v>
+      </c>
+      <c r="D25" s="3"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="4">
+        <v>7</v>
+      </c>
+      <c r="D26" s="3"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="4">
+        <v>7</v>
+      </c>
+      <c r="D27" s="3"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C28" s="4">
+        <v>7</v>
+      </c>
+      <c r="D28" s="3"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" s="4">
+        <v>12</v>
+      </c>
+      <c r="D29" s="3"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" s="4">
+        <v>7</v>
+      </c>
+      <c r="D30" s="3"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C31" s="4">
         <v>3</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>3</v>
-      </c>
-      <c r="B23" s="1" t="s">
+      <c r="D31" s="3"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C32" s="4">
+        <v>5</v>
+      </c>
+      <c r="D32" s="3"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C33" s="4">
+        <v>43</v>
+      </c>
+      <c r="D33" s="3"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C34" s="4">
         <v>8</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>3</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>3</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>3</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>3</v>
-      </c>
-      <c r="B27" s="1" t="s">
+      <c r="D34" s="3"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C35" s="4">
+        <v>15</v>
+      </c>
+      <c r="D35" s="3"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" s="4">
+        <v>11</v>
+      </c>
+      <c r="D36" s="3"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C37" s="4">
+        <v>5</v>
+      </c>
+      <c r="D37" s="3"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C38" s="4">
+        <v>4</v>
+      </c>
+      <c r="D38" s="3"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C39" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>40</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C40" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C41" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C42" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>40</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C43" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>40</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C44" s="1">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>40</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C45" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>40</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C46" s="1">
         <v>24</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>3</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C29" s="1" t="s">
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>3</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>3</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>3</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>3</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>3</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>3</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C36" s="1" t="s">
+      <c r="B47" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B37" s="1" t="s">
+      <c r="C47" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>40</v>
+      </c>
+      <c r="B48" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>3</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>3</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>3</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>3</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>3</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>3</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>3</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>3</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>3</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>3</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>3</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>47</v>
+      <c r="C48" s="1">
+        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>61</v>
+        <v>52</v>
+      </c>
+      <c r="C49" s="1">
+        <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C50" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C50" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>40</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C51" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>40</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C52" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>40</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C53" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>40</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C54" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>40</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C55" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>40</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C56" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C57" s="1">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>59</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C58" s="1">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>59</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C59" s="1">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>59</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C60" s="1">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>59</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C61" s="1">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>59</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C62" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>59</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C63" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>59</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C64" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>59</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C65" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>59</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C66" s="1">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>59</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C67" s="1">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>59</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C68" s="1">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>59</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C69" s="1">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>59</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C70" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>59</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C71" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>59</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C72" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>59</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C73" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>59</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C74" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>59</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C75" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>59</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C76" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>59</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C77" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>59</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C78" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>59</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C79" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>59</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C80" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>59</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C81" s="1">
         <v>50</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B52" s="1"/>
-      <c r="C52" s="1"/>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B53" s="1"/>
-      <c r="C53" s="1"/>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B54" s="1"/>
-      <c r="C54" s="1"/>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B55" s="1"/>
-      <c r="C55" s="1"/>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B56" s="1"/>
-      <c r="C56" s="1"/>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B57" s="1"/>
-      <c r="C57" s="1"/>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B58" s="1"/>
-      <c r="C58" s="1"/>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B59" s="1"/>
-      <c r="C59" s="1"/>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B60" s="1"/>
-      <c r="C60" s="1"/>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B61" s="1"/>
-      <c r="C61" s="1"/>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B62" s="1"/>
-      <c r="C62" s="1"/>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B63" s="1"/>
-      <c r="C63" s="1"/>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B64" s="1"/>
-      <c r="C64" s="1"/>
-    </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B65" s="1"/>
-      <c r="C65" s="1"/>
-    </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B66" s="1"/>
-      <c r="C66" s="1"/>
-    </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B67" s="1"/>
-      <c r="C67" s="1"/>
-    </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B68" s="1"/>
-      <c r="C68" s="1"/>
-    </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B69" s="1"/>
-      <c r="C69" s="1"/>
-    </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B70" s="1"/>
-      <c r="C70" s="1"/>
-    </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B71" s="1"/>
-      <c r="C71" s="1"/>
-    </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B72" s="1"/>
-      <c r="C72" s="1"/>
-    </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B73" s="1"/>
-      <c r="C73" s="1"/>
-    </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B74" s="1"/>
-      <c r="C74" s="1"/>
-    </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B75" s="1"/>
-      <c r="C75" s="1"/>
-    </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B76" s="1"/>
-      <c r="C76" s="1"/>
-    </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B77" s="1"/>
-      <c r="C77" s="1"/>
-    </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B78" s="1"/>
-      <c r="C78" s="1"/>
-    </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B79" s="1"/>
-      <c r="C79" s="1"/>
-    </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B80" s="1"/>
-      <c r="C80" s="1"/>
-    </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B81" s="1"/>
-      <c r="C81" s="1"/>
-    </row>
-    <row r="82" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B82" s="1"/>
-      <c r="C82" s="1"/>
-    </row>
-    <row r="83" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B83" s="1"/>
-      <c r="C83" s="1"/>
-    </row>
-    <row r="84" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B84" s="1"/>
-      <c r="C84" s="1"/>
-    </row>
-    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B85" s="1"/>
-      <c r="C85" s="1"/>
-    </row>
-    <row r="86" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B86" s="1"/>
-      <c r="C86" s="1"/>
-    </row>
-    <row r="87" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B87" s="1"/>
-      <c r="C87" s="1"/>
-    </row>
-    <row r="88" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B88" s="1"/>
-      <c r="C88" s="1"/>
-    </row>
-    <row r="89" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B89" s="1"/>
-      <c r="C89" s="1"/>
-    </row>
-    <row r="90" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B90" s="1"/>
-      <c r="C90" s="1"/>
-    </row>
-    <row r="91" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B91" s="1"/>
-      <c r="C91" s="1"/>
-    </row>
-    <row r="92" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>59</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C82" s="1">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>59</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C83" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>59</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C84" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>59</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C85" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>59</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C86" s="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>59</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C87" s="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>59</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C88" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>59</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C89" s="1">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>59</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C90" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>59</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C91" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
     </row>
-    <row r="93" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
     </row>
-    <row r="94" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
     </row>
-    <row r="95" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
     </row>
-    <row r="96" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
     </row>

</xml_diff>

<commit_message>
real data first test
</commit_message>
<xml_diff>
--- a/addresses/good_addresses.xlsx
+++ b/addresses/good_addresses.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="98">
   <si>
     <t>City</t>
   </si>
@@ -141,63 +141,6 @@
     <t xml:space="preserve">שבט זבולון </t>
   </si>
   <si>
-    <t>עפולה</t>
-  </si>
-  <si>
-    <t>קונטיקט 5</t>
-  </si>
-  <si>
-    <t>הזהבן 4</t>
-  </si>
-  <si>
-    <t>חיננית 13</t>
-  </si>
-  <si>
-    <t>חטפית 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">פנקס צבי 8 </t>
-  </si>
-  <si>
-    <t>צוקית 9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">הרצל 19 </t>
-  </si>
-  <si>
-    <t>עלית הנוער 8</t>
-  </si>
-  <si>
-    <t>רחוב הרצל 24</t>
-  </si>
-  <si>
-    <t>הבריגדה היהודית 11</t>
-  </si>
-  <si>
-    <t>אבן גבירול 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">זבוטינסקי 10 </t>
-  </si>
-  <si>
-    <t>הרוגי מלכות 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">עליית הנוער 9 </t>
-  </si>
-  <si>
-    <t>ראסל 10</t>
-  </si>
-  <si>
-    <t>ירקון 11</t>
-  </si>
-  <si>
-    <t>אבן גבירול 45</t>
-  </si>
-  <si>
-    <t>אבן גבירול 30</t>
-  </si>
-  <si>
     <t>רכסים</t>
   </si>
   <si>
@@ -265,6 +208,111 @@
   </si>
   <si>
     <t xml:space="preserve">הרב קוק </t>
+  </si>
+  <si>
+    <t xml:space="preserve">משה רבינו  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">צמח צדק  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">שבט יהודה  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">שבט אשר  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> שבט זבולון</t>
+  </si>
+  <si>
+    <t xml:space="preserve">יעקב אבינו </t>
+  </si>
+  <si>
+    <t xml:space="preserve">בעל התניא </t>
+  </si>
+  <si>
+    <t xml:space="preserve">שבט אפרים </t>
+  </si>
+  <si>
+    <t xml:space="preserve">שבטי ישראל </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הרב עובדיה יוסף </t>
+  </si>
+  <si>
+    <t xml:space="preserve">משה רבנו </t>
+  </si>
+  <si>
+    <t xml:space="preserve">יצחק אבינו </t>
+  </si>
+  <si>
+    <t>חתם סופר</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>שדי חמד</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>אור החיים</t>
+  </si>
+  <si>
+    <t>חזון דוד</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>נתיבות המשפט</t>
+  </si>
+  <si>
+    <t>93</t>
+  </si>
+  <si>
+    <t>מסילת יוסף</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>85</t>
+  </si>
+  <si>
+    <t>משך חכמה</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>שאגת אריה</t>
+  </si>
+  <si>
+    <t>רמבם</t>
+  </si>
+  <si>
+    <t>71</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>אבני נזר</t>
+  </si>
+  <si>
+    <t>מסילת ישרים</t>
+  </si>
+  <si>
+    <t>40</t>
   </si>
 </sst>
 </file>
@@ -314,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -328,6 +376,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -631,12 +682,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E261"/>
+  <dimension ref="A1:H261"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.8984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.59765625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.3984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -864,244 +916,254 @@
       <c r="D20" s="3"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C21" s="4">
-        <v>46</v>
+      <c r="A21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>15</v>
       </c>
       <c r="D21" s="3"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C22" s="4">
-        <v>6</v>
+      <c r="A22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>76</v>
       </c>
       <c r="D22" s="3"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C23" s="4">
-        <v>3</v>
+      <c r="A23" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>78</v>
       </c>
       <c r="D23" s="3"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C24" s="4">
-        <v>8</v>
+      <c r="A24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="D24" s="3"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C25" s="4">
+      <c r="A25" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D25" s="3"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="3"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D27" s="3"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D28" s="3"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D29" s="3"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>3</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D30" s="3"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D31" s="3"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D32" s="3"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>3</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D33" s="3"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>3</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D25" s="3"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C26" s="4">
-        <v>7</v>
-      </c>
-      <c r="D26" s="3"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C27" s="4">
-        <v>7</v>
-      </c>
-      <c r="D27" s="3"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C28" s="4">
-        <v>7</v>
-      </c>
-      <c r="D28" s="3"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C29" s="4">
-        <v>12</v>
-      </c>
-      <c r="D29" s="3"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C30" s="4">
-        <v>7</v>
-      </c>
-      <c r="D30" s="3"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C31" s="4">
-        <v>3</v>
-      </c>
-      <c r="D31" s="3"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C32" s="4">
-        <v>5</v>
-      </c>
-      <c r="D32" s="3"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C33" s="4">
-        <v>43</v>
-      </c>
-      <c r="D33" s="3"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C34" s="4">
-        <v>8</v>
-      </c>
       <c r="D34" s="3"/>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C35" s="4">
-        <v>15</v>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>3</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="D35" s="3"/>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C36" s="4">
-        <v>11</v>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>26</v>
       </c>
       <c r="D36" s="3"/>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C37" s="4">
-        <v>5</v>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>93</v>
       </c>
       <c r="D37" s="3"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C38" s="4">
-        <v>4</v>
+      <c r="F37" s="3"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="4"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>3</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>94</v>
       </c>
       <c r="D38" s="3"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F38" s="3"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C39" s="1">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C40" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>40</v>
       </c>
@@ -1109,704 +1171,897 @@
         <v>41</v>
       </c>
       <c r="C41" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>40</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C42" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>40</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C43" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+      <c r="G43" s="1"/>
+      <c r="H43" s="1"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>40</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C44" s="1">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>40</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C45" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+      <c r="G45" s="1"/>
+      <c r="H45" s="1"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>40</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C46" s="1">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>40</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="C47" s="1">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>40</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C48" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>40</v>
       </c>
       <c r="B49" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C49" s="1">
+        <v>5</v>
+      </c>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>40</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C50" s="1">
+        <v>28</v>
+      </c>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>40</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C51" s="1">
+        <v>24</v>
+      </c>
+      <c r="G51" s="1"/>
+      <c r="H51" s="1"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>40</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C52" s="1">
+        <v>38</v>
+      </c>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>40</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C53" s="1">
+        <v>36</v>
+      </c>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>40</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C54" s="1">
+        <v>32</v>
+      </c>
+      <c r="G54" s="1"/>
+      <c r="H54" s="1"/>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>40</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C55" s="1">
+        <v>13</v>
+      </c>
+      <c r="G55" s="1"/>
+      <c r="H55" s="1"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>40</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C56" s="1">
+        <v>13</v>
+      </c>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>40</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C57" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>40</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C58" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>40</v>
+      </c>
+      <c r="B59" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C49" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>40</v>
-      </c>
-      <c r="B50" s="1" t="s">
+      <c r="C59" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>40</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C50" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>40</v>
-      </c>
-      <c r="B51" s="1" t="s">
+      <c r="C60" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>40</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C51" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>40</v>
-      </c>
-      <c r="B52" s="1" t="s">
+      <c r="C61" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>40</v>
+      </c>
+      <c r="B62" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C52" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>40</v>
-      </c>
-      <c r="B53" s="1" t="s">
+      <c r="C62" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>40</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C53" s="1">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>40</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C54" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>40</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C55" s="1">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>40</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C56" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>59</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C57" s="1">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>59</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C58" s="1">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>59</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C59" s="1">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>59</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C60" s="1">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>59</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C61" s="1">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>59</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C62" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>59</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="C63" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C64" s="1">
-        <v>4</v>
+        <v>40</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="C65" s="1">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>40</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C66" s="1">
         <v>59</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C66" s="1">
-        <v>28</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="C67" s="1">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C68" s="1">
-        <v>38</v>
+        <v>8</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>40</v>
+      </c>
+      <c r="B69" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B69" s="1" t="s">
-        <v>67</v>
-      </c>
       <c r="C69" s="1">
-        <v>36</v>
+        <v>15</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C70" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="C71" s="1">
-        <v>13</v>
+        <v>26</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C72" s="1">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="C73" s="1">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C74" s="1">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="B75" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C75" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B76" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C76" s="4">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B77" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C77" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B78" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C78" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B79" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C79" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B80" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C80" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B81" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C81" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B82" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C82" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B83" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C83" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B84" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C84" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C85" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B86" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C86" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B87" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C87" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B88" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C88" s="4">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B89" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C89" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B90" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C90" s="4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B91" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C91" s="4">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C92" s="6">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C93" s="6">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C94" s="6">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C95" s="6">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C96" s="6">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C97" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C98" s="6">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C99" s="6">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B100" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C75" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>59</v>
-      </c>
-      <c r="B76" s="1" t="s">
+      <c r="C100" s="6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C101" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C102" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C103" s="6">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B104" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C76" s="1">
+      <c r="C104" s="6">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C105" s="6">
         <v>5</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>59</v>
-      </c>
-      <c r="B77" s="1" t="s">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C106" s="6">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A107" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C107" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C108" s="6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C109" s="6">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B110" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C77" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>59</v>
-      </c>
-      <c r="B78" s="1" t="s">
+      <c r="C110" s="6">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C111" s="6">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B112" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C78" s="1">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>59</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C79" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>59</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C80" s="1">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>59</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C81" s="1">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>59</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C82" s="1">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>59</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C83" s="1">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>59</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C84" s="1">
+      <c r="C112" s="6">
         <v>8</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>59</v>
-      </c>
-      <c r="B85" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C85" s="1">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>59</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C86" s="1">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>59</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C87" s="1">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>59</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C88" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>59</v>
-      </c>
-      <c r="B89" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C89" s="1">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>59</v>
-      </c>
-      <c r="B90" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C90" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>59</v>
-      </c>
-      <c r="B91" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C91" s="1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B92" s="1"/>
-      <c r="C92" s="1"/>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B93" s="1"/>
-      <c r="C93" s="1"/>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B94" s="1"/>
-      <c r="C94" s="1"/>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B95" s="1"/>
-      <c r="C95" s="1"/>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B96" s="1"/>
-      <c r="C96" s="1"/>
-    </row>
-    <row r="97" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B97" s="1"/>
-      <c r="C97" s="1"/>
-    </row>
-    <row r="98" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B98" s="1"/>
-      <c r="C98" s="1"/>
-    </row>
-    <row r="99" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B99" s="1"/>
-      <c r="C99" s="1"/>
-    </row>
-    <row r="100" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B100" s="1"/>
-      <c r="C100" s="1"/>
-    </row>
-    <row r="101" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B101" s="1"/>
-      <c r="C101" s="1"/>
-    </row>
-    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B102" s="1"/>
-      <c r="C102" s="1"/>
-    </row>
-    <row r="103" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B103" s="1"/>
-      <c r="C103" s="1"/>
-    </row>
-    <row r="104" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B104" s="1"/>
-      <c r="C104" s="1"/>
-    </row>
-    <row r="105" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B105" s="1"/>
-      <c r="C105" s="1"/>
-    </row>
-    <row r="106" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B106" s="1"/>
-      <c r="C106" s="1"/>
-    </row>
-    <row r="107" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B107" s="1"/>
-      <c r="C107" s="1"/>
-    </row>
-    <row r="108" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B108" s="1"/>
-      <c r="C108" s="1"/>
-    </row>
-    <row r="109" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B109" s="1"/>
-      <c r="C109" s="1"/>
-    </row>
-    <row r="110" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B110" s="1"/>
-      <c r="C110" s="1"/>
-    </row>
-    <row r="111" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B111" s="1"/>
-      <c r="C111" s="1"/>
-    </row>
-    <row r="112" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B112" s="1"/>
-      <c r="C112" s="1"/>
-    </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B113" s="1"/>
-      <c r="C113" s="1"/>
-    </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B114" s="1"/>
-      <c r="C114" s="1"/>
-    </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C113" s="6">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A114" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C114" s="6">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
     </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
     </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
     </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
     </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B119" s="1"/>
       <c r="C119" s="1"/>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B120" s="1"/>
       <c r="C120" s="1"/>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B121" s="1"/>
       <c r="C121" s="1"/>
     </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
     </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B123" s="1"/>
       <c r="C123" s="1"/>
     </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
     </row>
-    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
     </row>
-    <row r="126" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
     </row>
-    <row r="127" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B127" s="1"/>
       <c r="C127" s="1"/>
     </row>
-    <row r="128" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
     </row>

</xml_diff>